<commit_message>
docs(amphion-asr): expand whispered-speech ASR table with 9 baselines - Table 16: add Whisper/Kimi/Step-Audio2/MiniCPM-o/MOSS-Audio/Qwen3/   FireRed/GLM-ASR-nano/Fun-ASR-Nano results from audiollm-eval whisp runs - AmphionASR lowest on both wEar (zh, 0.58 CER) and WTIMIT (en, 6.11 WER) - Drop redundant CER/WER suffixes from column headers (caption covers it) - Add cross-system analysis paragraph - Fill data.xlsx Whisper-ASR sheet with all comparison models - Fix Gemini 3-Flash citation in noise-robustness section - Markdown formatting cleanup in paper-review notes
</commit_message>
<xml_diff>
--- a/egs/amphion-asr-1.7b-2026/refs/docs/data.xlsx
+++ b/egs/amphion-asr-1.7b-2026/refs/docs/data.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
   <sheets>
     <sheet name="ASR" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="ASR-hotwords" sheetId="2" state="visible" r:id="rId2"/>
@@ -12,27 +12,37 @@
     <sheet name="Whisper-ASR" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,13 +57,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -452,7 +471,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -541,30 +563,22 @@
           <t>1.88 | 3.68</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="C3" t="n">
+        <v>10</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>9.98 | 19.00</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>5.59</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>5.23</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>29.03</t>
-        </is>
+      <c r="E3" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G3" t="n">
+        <v>29.03</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -583,30 +597,22 @@
           <t>1.61 | 3.39</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>8.68</t>
-        </is>
+      <c r="C4" t="n">
+        <v>8.68</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>5.04 | 5.85</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>1.58</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2.77</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>5.21</t>
-        </is>
+      <c r="E4" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5.21</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -625,30 +631,22 @@
           <t>1.30｜2.56</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>9.59</t>
-        </is>
+      <c r="C5" t="n">
+        <v>9.59</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>5.82｜6.03</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>0.81</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2.62</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>5.36</t>
-        </is>
+      <c r="E5" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5.36</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -667,30 +665,22 @@
           <t>1.43｜ 2.98</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>9.19</t>
-        </is>
+      <c r="C6" t="n">
+        <v>9.19</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>4.43 | 4.49</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>0.65</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2.37</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>3.19</t>
-        </is>
+      <c r="E6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3.19</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -709,30 +699,22 @@
           <t>4.66 | 7.26</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>8.96</t>
-        </is>
+      <c r="C7" t="n">
+        <v>8.960000000000001</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>5.97 | 7.61</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2.31</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>3.05</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>14.97</t>
-        </is>
+      <c r="E7" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="G7" t="n">
+        <v>14.97</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -751,30 +733,22 @@
           <t>2.13 | 4.42</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>9.43</t>
-        </is>
+      <c r="C8" t="n">
+        <v>9.43</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>6.43 | 8.54</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>3.53</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>9.36</t>
-        </is>
+      <c r="E8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="G8" t="n">
+        <v>9.359999999999999</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -788,15 +762,11 @@
           <t>Mimo-Audio</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>1.97</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>6.71</t>
-        </is>
+      <c r="E9" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6.71</v>
       </c>
     </row>
     <row r="10">
@@ -810,30 +780,22 @@
           <t>1.41 ｜ 2.75</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>9.9</t>
-        </is>
+      <c r="C10" t="n">
+        <v>9.9</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>5.40 | 5.51</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>0.83</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2.35</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>4.16</t>
-        </is>
+      <c r="E10" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.16</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -852,30 +814,22 @@
           <t>1.46 | 3.57</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>9.31</t>
-        </is>
+      <c r="C11" t="n">
+        <v>9.31</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>6.14 | 7.10</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>1.05</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2.91</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>7.65</t>
-        </is>
+      <c r="E11" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="G11" t="n">
+        <v>7.65</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -884,7 +838,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -894,8 +849,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:N28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1022,7 +980,6 @@
         <v>7.413329595984048</v>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -1185,7 +1142,6 @@
         <v>6.385133843821269</v>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1249,20 +1205,14 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>10646</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>7.05</t>
-        </is>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>10646</v>
+      </c>
+      <c r="K10" t="n">
+        <v>7.05</v>
       </c>
     </row>
     <row r="11">
@@ -1271,50 +1221,32 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>8.19</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>69.34</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>3.83</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>4.85</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>91.81</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>95.66</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>10647</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>4.55</t>
-        </is>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>8.19</v>
+      </c>
+      <c r="E11" t="n">
+        <v>69.34</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4.85</v>
+      </c>
+      <c r="H11" t="n">
+        <v>91.81</v>
+      </c>
+      <c r="I11" t="n">
+        <v>95.66</v>
+      </c>
+      <c r="J11" t="n">
+        <v>10647</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4.55</v>
       </c>
     </row>
     <row r="12">
@@ -1323,50 +1255,32 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>12.11</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>67.01</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>5.16</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>4.76</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>87.89</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>93.46</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>10646</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>4.88</t>
-        </is>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" t="n">
+        <v>12.11</v>
+      </c>
+      <c r="E12" t="n">
+        <v>67.01000000000001</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5.16</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="H12" t="n">
+        <v>87.89</v>
+      </c>
+      <c r="I12" t="n">
+        <v>93.45999999999999</v>
+      </c>
+      <c r="J12" t="n">
+        <v>10646</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4.88</v>
       </c>
     </row>
     <row r="13">
@@ -1375,50 +1289,32 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>15.48</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>64.26</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>6.36</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>4.74</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>84.52</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>91.51</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>10647</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>5.22</t>
-        </is>
+      <c r="C13" t="n">
+        <v>15</v>
+      </c>
+      <c r="D13" t="n">
+        <v>15.48</v>
+      </c>
+      <c r="E13" t="n">
+        <v>64.26000000000001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6.36</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="H13" t="n">
+        <v>84.52</v>
+      </c>
+      <c r="I13" t="n">
+        <v>91.51000000000001</v>
+      </c>
+      <c r="J13" t="n">
+        <v>10647</v>
+      </c>
+      <c r="K13" t="n">
+        <v>5.22</v>
       </c>
     </row>
     <row r="14">
@@ -1427,50 +1323,32 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>18.78</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>62.35</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>7.59</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>4.67</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>81.22</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>89.52</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>10647</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>5.53</t>
-        </is>
+      <c r="C14" t="n">
+        <v>20</v>
+      </c>
+      <c r="D14" t="n">
+        <v>18.78</v>
+      </c>
+      <c r="E14" t="n">
+        <v>62.35</v>
+      </c>
+      <c r="F14" t="n">
+        <v>7.59</v>
+      </c>
+      <c r="G14" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="H14" t="n">
+        <v>81.22</v>
+      </c>
+      <c r="I14" t="n">
+        <v>89.52</v>
+      </c>
+      <c r="J14" t="n">
+        <v>10647</v>
+      </c>
+      <c r="K14" t="n">
+        <v>5.53</v>
       </c>
     </row>
     <row r="15">
@@ -1479,20 +1357,14 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>16293</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>11.32</t>
-        </is>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>16293</v>
+      </c>
+      <c r="K15" t="n">
+        <v>11.32</v>
       </c>
     </row>
     <row r="16">
@@ -1501,50 +1373,32 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>15.59</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>60.81</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>11.59</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>9.26</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>84.41</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>90.55</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>16289</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>9.46</t>
-        </is>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="E16" t="n">
+        <v>60.81</v>
+      </c>
+      <c r="F16" t="n">
+        <v>11.59</v>
+      </c>
+      <c r="G16" t="n">
+        <v>9.26</v>
+      </c>
+      <c r="H16" t="n">
+        <v>84.41</v>
+      </c>
+      <c r="I16" t="n">
+        <v>90.55</v>
+      </c>
+      <c r="J16" t="n">
+        <v>16289</v>
+      </c>
+      <c r="K16" t="n">
+        <v>9.460000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1553,50 +1407,32 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>19.33</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>59.74</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>13.73</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>9.33</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>80.67</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>88.34</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>16292</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>9.73</t>
-        </is>
+      <c r="C17" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" t="n">
+        <v>19.33</v>
+      </c>
+      <c r="E17" t="n">
+        <v>59.74</v>
+      </c>
+      <c r="F17" t="n">
+        <v>13.73</v>
+      </c>
+      <c r="G17" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="H17" t="n">
+        <v>80.67</v>
+      </c>
+      <c r="I17" t="n">
+        <v>88.34</v>
+      </c>
+      <c r="J17" t="n">
+        <v>16292</v>
+      </c>
+      <c r="K17" t="n">
+        <v>9.73</v>
       </c>
     </row>
     <row r="18">
@@ -1605,50 +1441,32 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>23.79</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>58.34</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>16.68</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>9.4</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>76.21</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>85.79</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>16293</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>10.05</t>
-        </is>
+      <c r="C18" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" t="n">
+        <v>23.79</v>
+      </c>
+      <c r="E18" t="n">
+        <v>58.34</v>
+      </c>
+      <c r="F18" t="n">
+        <v>16.68</v>
+      </c>
+      <c r="G18" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H18" t="n">
+        <v>76.20999999999999</v>
+      </c>
+      <c r="I18" t="n">
+        <v>85.79000000000001</v>
+      </c>
+      <c r="J18" t="n">
+        <v>16293</v>
+      </c>
+      <c r="K18" t="n">
+        <v>10.05</v>
       </c>
     </row>
     <row r="19">
@@ -1657,50 +1475,32 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>26.6</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>57.88</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>9.42</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>73.4</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>84.02</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>16293</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>10.28</t>
-        </is>
+      <c r="C19" t="n">
+        <v>20</v>
+      </c>
+      <c r="D19" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>57.88</v>
+      </c>
+      <c r="F19" t="n">
+        <v>19</v>
+      </c>
+      <c r="G19" t="n">
+        <v>9.42</v>
+      </c>
+      <c r="H19" t="n">
+        <v>73.40000000000001</v>
+      </c>
+      <c r="I19" t="n">
+        <v>84.02</v>
+      </c>
+      <c r="J19" t="n">
+        <v>16293</v>
+      </c>
+      <c r="K19" t="n">
+        <v>10.28</v>
       </c>
     </row>
     <row r="20">
@@ -1776,60 +1576,38 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>37.94</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>49.39</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>16.95</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>5.51</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>62.06</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>75.88</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>10645</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>8.89</t>
-        </is>
+      <c r="C21" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F21" t="n">
+        <v>37.94</v>
+      </c>
+      <c r="G21" t="n">
+        <v>49.39</v>
+      </c>
+      <c r="H21" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="J21" t="n">
+        <v>62.06</v>
+      </c>
+      <c r="K21" t="n">
+        <v>75.88</v>
+      </c>
+      <c r="L21" t="n">
+        <v>10645</v>
+      </c>
+      <c r="M21" t="n">
+        <v>8.890000000000001</v>
       </c>
     </row>
     <row r="22">
@@ -1838,60 +1616,38 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>0.08</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>0.06</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>37.55</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>49.6</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>16.42</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>5.57</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>62.45</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>76.23</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>10644</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>8.77</t>
-        </is>
+      <c r="C22" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F22" t="n">
+        <v>37.55</v>
+      </c>
+      <c r="G22" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="H22" t="n">
+        <v>16.42</v>
+      </c>
+      <c r="I22" t="n">
+        <v>5.57</v>
+      </c>
+      <c r="J22" t="n">
+        <v>62.45</v>
+      </c>
+      <c r="K22" t="n">
+        <v>76.23</v>
+      </c>
+      <c r="L22" t="n">
+        <v>10644</v>
+      </c>
+      <c r="M22" t="n">
+        <v>8.77</v>
       </c>
     </row>
     <row r="23">
@@ -1900,60 +1656,38 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>35.98</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>50.91</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>14.83</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>5.05</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>64.02</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>77.88</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>10647</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>7.94</t>
-        </is>
+      <c r="C23" t="n">
+        <v>15</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="F23" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="G23" t="n">
+        <v>50.91</v>
+      </c>
+      <c r="H23" t="n">
+        <v>14.83</v>
+      </c>
+      <c r="I23" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="J23" t="n">
+        <v>64.02</v>
+      </c>
+      <c r="K23" t="n">
+        <v>77.88</v>
+      </c>
+      <c r="L23" t="n">
+        <v>10647</v>
+      </c>
+      <c r="M23" t="n">
+        <v>7.94</v>
       </c>
     </row>
     <row r="24">
@@ -1962,60 +1696,38 @@
           <t>commonvoice_zh_hotwords</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>0.17</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>35.69</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>51.5</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>14.67</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>4.93</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>64.31</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>78.14</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>10647</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>7.8</t>
-        </is>
+      <c r="C24" t="n">
+        <v>20</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>35.69</v>
+      </c>
+      <c r="G24" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="H24" t="n">
+        <v>14.67</v>
+      </c>
+      <c r="I24" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="J24" t="n">
+        <v>64.31</v>
+      </c>
+      <c r="K24" t="n">
+        <v>78.14</v>
+      </c>
+      <c r="L24" t="n">
+        <v>10647</v>
+      </c>
+      <c r="M24" t="n">
+        <v>7.8</v>
       </c>
     </row>
     <row r="25">
@@ -2024,60 +1736,38 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>0.06</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>47.15</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>51.76</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>34.76</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>10.03</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>52.85</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>68.71</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>16294</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>12.23</t>
-        </is>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F25" t="n">
+        <v>47.15</v>
+      </c>
+      <c r="G25" t="n">
+        <v>51.76</v>
+      </c>
+      <c r="H25" t="n">
+        <v>34.76</v>
+      </c>
+      <c r="I25" t="n">
+        <v>10.03</v>
+      </c>
+      <c r="J25" t="n">
+        <v>52.85</v>
+      </c>
+      <c r="K25" t="n">
+        <v>68.70999999999999</v>
+      </c>
+      <c r="L25" t="n">
+        <v>16294</v>
+      </c>
+      <c r="M25" t="n">
+        <v>12.23</v>
       </c>
     </row>
     <row r="26">
@@ -2086,60 +1776,38 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>0.13</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>48.88</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>51.03</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>39.61</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>10.26</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>51.12</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>66.7</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>16289</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>12.88</t>
-        </is>
+      <c r="C26" t="n">
+        <v>10</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F26" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="G26" t="n">
+        <v>51.03</v>
+      </c>
+      <c r="H26" t="n">
+        <v>39.61</v>
+      </c>
+      <c r="I26" t="n">
+        <v>10.26</v>
+      </c>
+      <c r="J26" t="n">
+        <v>51.12</v>
+      </c>
+      <c r="K26" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="L26" t="n">
+        <v>16289</v>
+      </c>
+      <c r="M26" t="n">
+        <v>12.88</v>
       </c>
     </row>
     <row r="27">
@@ -2148,60 +1816,38 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>0.19</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>50.37</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>50.85</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>39.37</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>10.32</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>49.63</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>65.16</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>16292</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>12.9</t>
-        </is>
+      <c r="C27" t="n">
+        <v>15</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F27" t="n">
+        <v>50.37</v>
+      </c>
+      <c r="G27" t="n">
+        <v>50.85</v>
+      </c>
+      <c r="H27" t="n">
+        <v>39.37</v>
+      </c>
+      <c r="I27" t="n">
+        <v>10.32</v>
+      </c>
+      <c r="J27" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="K27" t="n">
+        <v>65.16</v>
+      </c>
+      <c r="L27" t="n">
+        <v>16292</v>
+      </c>
+      <c r="M27" t="n">
+        <v>12.9</v>
       </c>
     </row>
     <row r="28">
@@ -2210,77 +1856,43 @@
           <t>commonvoice_en_hotwords</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>0.27</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>50.23</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>50.95</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>37.41</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>10.04</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>49.77</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>65.73</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>16291</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>12.48</t>
-        </is>
-      </c>
-    </row>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
+      <c r="C28" t="n">
+        <v>20</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F28" t="n">
+        <v>50.23</v>
+      </c>
+      <c r="G28" t="n">
+        <v>50.95</v>
+      </c>
+      <c r="H28" t="n">
+        <v>37.41</v>
+      </c>
+      <c r="I28" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="J28" t="n">
+        <v>49.77</v>
+      </c>
+      <c r="K28" t="n">
+        <v>65.73</v>
+      </c>
+      <c r="L28" t="n">
+        <v>16291</v>
+      </c>
+      <c r="M28" t="n">
+        <v>12.48</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -2291,9 +1903,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
+  </cols>
   <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -2304,7 +1920,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="E1" t="inlineStr">
@@ -2366,10 +1985,8 @@
           <t>cv-en-test</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>16402</t>
-        </is>
+      <c r="B3" t="n">
+        <v>16402</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -2381,20 +1998,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>11.54</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>12.33</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>11.61</t>
-        </is>
+      <c r="E3" t="n">
+        <v>11.54</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12.33</v>
+      </c>
+      <c r="G3" t="n">
+        <v>11.61</v>
       </c>
     </row>
     <row r="4">
@@ -2408,20 +2019,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>12.36</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>13.41</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>12.27</t>
-        </is>
+      <c r="E4" t="n">
+        <v>12.36</v>
+      </c>
+      <c r="F4" t="n">
+        <v>13.41</v>
+      </c>
+      <c r="G4" t="n">
+        <v>12.27</v>
       </c>
     </row>
     <row r="5">
@@ -2435,20 +2040,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>11.57</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>11.21</t>
-        </is>
+      <c r="E5" t="n">
+        <v>11</v>
+      </c>
+      <c r="F5" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="G5" t="n">
+        <v>11.21</v>
       </c>
     </row>
     <row r="6">
@@ -2462,20 +2061,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>9.84</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>10.84</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>10.43</t>
-        </is>
+      <c r="E6" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="G6" t="n">
+        <v>10.43</v>
       </c>
     </row>
     <row r="7">
@@ -2489,20 +2082,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>9.92</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>10.58</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>10.31</t>
-        </is>
+      <c r="E7" t="n">
+        <v>9.92</v>
+      </c>
+      <c r="F7" t="n">
+        <v>10.58</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10.31</v>
       </c>
     </row>
     <row r="8">
@@ -2516,20 +2103,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>26.53</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>41.19</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>18.74</t>
-        </is>
+      <c r="E8" t="n">
+        <v>26.53</v>
+      </c>
+      <c r="F8" t="n">
+        <v>41.19</v>
+      </c>
+      <c r="G8" t="n">
+        <v>18.74</v>
       </c>
     </row>
     <row r="9">
@@ -2543,20 +2124,14 @@
           <t>rir</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>9.71</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>10.77</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>10.59</t>
-        </is>
+      <c r="E9" t="n">
+        <v>9.710000000000001</v>
+      </c>
+      <c r="F9" t="n">
+        <v>10.77</v>
+      </c>
+      <c r="G9" t="n">
+        <v>10.59</v>
       </c>
     </row>
     <row r="10">
@@ -2570,20 +2145,14 @@
           <t>rir</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>27.47</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>29.66</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>29.07</t>
-        </is>
+      <c r="E10" t="n">
+        <v>27.47</v>
+      </c>
+      <c r="F10" t="n">
+        <v>29.66</v>
+      </c>
+      <c r="G10" t="n">
+        <v>29.07</v>
       </c>
     </row>
     <row r="11">
@@ -2597,20 +2166,14 @@
           <t>rir</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>14.16</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>15.6</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>15.23</t>
-        </is>
+      <c r="E11" t="n">
+        <v>14.16</v>
+      </c>
+      <c r="F11" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G11" t="n">
+        <v>15.23</v>
       </c>
     </row>
     <row r="12">
@@ -2624,20 +2187,14 @@
           <t>rir</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>10.91</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>12.22</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>12.11</t>
-        </is>
+      <c r="E12" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="F12" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12.11</v>
       </c>
     </row>
     <row r="13">
@@ -2651,20 +2208,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>11.12</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>11.63</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>11.47</t>
-        </is>
+      <c r="E13" t="n">
+        <v>11.12</v>
+      </c>
+      <c r="F13" t="n">
+        <v>11.63</v>
+      </c>
+      <c r="G13" t="n">
+        <v>11.47</v>
       </c>
     </row>
     <row r="15">
@@ -2673,10 +2224,8 @@
           <t>cv-zh-test</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>10647</t>
-        </is>
+      <c r="B15" t="n">
+        <v>10647</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -2688,20 +2237,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>6.4</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>7.67</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>7.34</t>
-        </is>
+      <c r="E15" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F15" t="n">
+        <v>7.67</v>
+      </c>
+      <c r="G15" t="n">
+        <v>7.34</v>
       </c>
     </row>
     <row r="16">
@@ -2715,20 +2258,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>6.75</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>8.1</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>7.62</t>
-        </is>
+      <c r="E16" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>7.62</v>
       </c>
     </row>
     <row r="17">
@@ -2742,20 +2279,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>6.25</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>7.5</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>7.28</t>
-        </is>
+      <c r="E17" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F17" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G17" t="n">
+        <v>7.28</v>
       </c>
     </row>
     <row r="18">
@@ -2769,20 +2300,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>6.05</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>7.06</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>6.95</t>
-        </is>
+      <c r="E18" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="F18" t="n">
+        <v>7.06</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6.95</v>
       </c>
     </row>
     <row r="19">
@@ -2796,20 +2321,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>5.87</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>7.02</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>6.9</t>
-        </is>
+      <c r="E19" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="F19" t="n">
+        <v>7.02</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6.9</v>
       </c>
     </row>
     <row r="20">
@@ -2823,20 +2342,14 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>19.9</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>21.45</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>9.45</t>
-        </is>
+      <c r="E20" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="F20" t="n">
+        <v>21.45</v>
+      </c>
+      <c r="G20" t="n">
+        <v>9.449999999999999</v>
       </c>
     </row>
     <row r="21">
@@ -2850,20 +2363,14 @@
           <t>rir</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>5.75</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>6.9</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>6.82</t>
-        </is>
+      <c r="E21" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G21" t="n">
+        <v>6.82</v>
       </c>
     </row>
     <row r="22">
@@ -2877,20 +2384,14 @@
           <t>rir</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>16.62</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>19.89</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>19.71</t>
-        </is>
+      <c r="E22" t="n">
+        <v>16.62</v>
+      </c>
+      <c r="F22" t="n">
+        <v>19.89</v>
+      </c>
+      <c r="G22" t="n">
+        <v>19.71</v>
       </c>
     </row>
     <row r="23">
@@ -2904,20 +2405,14 @@
           <t>rir</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>9.31</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>10.95</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>10.89</t>
-        </is>
+      <c r="E23" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="F23" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="G23" t="n">
+        <v>10.89</v>
       </c>
     </row>
     <row r="24">
@@ -2931,20 +2426,14 @@
           <t>rir</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>6.39</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>7.72</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>7.6</t>
-        </is>
+      <c r="E24" t="n">
+        <v>6.39</v>
+      </c>
+      <c r="F24" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="G24" t="n">
+        <v>7.6</v>
       </c>
     </row>
     <row r="25">
@@ -2958,24 +2447,19 @@
           <t>noise(5~20db)</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>6.43</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>7.66</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>7.47</t>
-        </is>
+      <c r="E25" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="F25" t="n">
+        <v>7.66</v>
+      </c>
+      <c r="G25" t="n">
+        <v>7.47</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -2986,7 +2470,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3051,53 +2538,35 @@
           <t>vitw_real_noise</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="B2" t="n">
+        <v>150</v>
       </c>
       <c r="C2" t="n">
         <v>6.64</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>6.12</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>7.51</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>7.63</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>8.21</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>13.19</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>16.57</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>11.92</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>35.1</t>
-        </is>
+      <c r="D2" t="n">
+        <v>6.12</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7.51</v>
+      </c>
+      <c r="F2" t="n">
+        <v>7.63</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="H2" t="n">
+        <v>13.19</v>
+      </c>
+      <c r="I2" t="n">
+        <v>16.57</v>
+      </c>
+      <c r="J2" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="K2" t="n">
+        <v>35.1</v>
       </c>
     </row>
     <row r="3">
@@ -3106,53 +2575,35 @@
           <t>vitw_real_far_field</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="B3" t="n">
+        <v>150</v>
       </c>
       <c r="C3" t="n">
         <v>2.27</v>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2.33</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2.23</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>5.14</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>3.06</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>1.87</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>3.38</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2.35</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>2.71</t>
-        </is>
+      <c r="D3" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.23</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5.14</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="K3" t="n">
+        <v>2.71</v>
       </c>
     </row>
     <row r="4">
@@ -3161,48 +2612,32 @@
           <t>vitw_real_echo</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="B4" t="n">
+        <v>150</v>
       </c>
       <c r="C4" t="n">
         <v>7.91</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>8.66</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>10.4</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>8.75</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>16.55</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>15.62</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>25.34</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>20.01</t>
-        </is>
+      <c r="D4" t="n">
+        <v>8.66</v>
+      </c>
+      <c r="E4" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="H4" t="n">
+        <v>15.62</v>
+      </c>
+      <c r="I4" t="n">
+        <v>25.34</v>
+      </c>
+      <c r="J4" t="n">
+        <v>20.01</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -3216,53 +2651,35 @@
           <t>vitw_real_distortion</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="B5" t="n">
+        <v>150</v>
       </c>
       <c r="C5" t="n">
         <v>1.92</v>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>1.54</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>3.15</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>3.89</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>3.7</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>3.74</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2.46</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>1.83</t>
-        </is>
+      <c r="D5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="J5" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1.83</v>
       </c>
     </row>
     <row r="6">
@@ -3271,53 +2688,35 @@
           <t>vitw_real_mixed</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>450</t>
-        </is>
+      <c r="B6" t="n">
+        <v>450</v>
       </c>
       <c r="C6" t="n">
         <v>2.85</v>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2.63</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>3.3</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>7.99</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>6.88</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>5.62</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>8.91</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>6.4</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>4.44</t>
-        </is>
+      <c r="D6" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="I6" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="J6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4.44</v>
       </c>
     </row>
     <row r="7">
@@ -3326,53 +2725,35 @@
           <t>vitw_real_obstructed</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="B7" t="n">
+        <v>150</v>
       </c>
       <c r="C7" t="n">
         <v>1.38</v>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>1.73</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>3.73</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>1.57</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>3.06</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>2.49</t>
-        </is>
+      <c r="D7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3.06</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K7" t="n">
+        <v>2.49</v>
       </c>
     </row>
     <row r="8">
@@ -3381,53 +2762,35 @@
           <t>vitw_real_recording</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="B8" t="n">
+        <v>150</v>
       </c>
       <c r="C8" t="n">
         <v>6.32</v>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>6.91</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>9.57</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>8.38</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>18.48</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>13.37</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>18.33</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>13.71</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>8.73</t>
-        </is>
+      <c r="D8" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="F8" t="n">
+        <v>8.380000000000001</v>
+      </c>
+      <c r="G8" t="n">
+        <v>18.48</v>
+      </c>
+      <c r="H8" t="n">
+        <v>13.37</v>
+      </c>
+      <c r="I8" t="n">
+        <v>18.33</v>
+      </c>
+      <c r="J8" t="n">
+        <v>13.71</v>
+      </c>
+      <c r="K8" t="n">
+        <v>8.73</v>
       </c>
     </row>
     <row r="9">
@@ -3436,53 +2799,35 @@
           <t>vitw_real_dropout</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
+      <c r="B9" t="n">
+        <v>150</v>
       </c>
       <c r="C9" t="n">
         <v>2.32</v>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2.72</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>4.16</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>5.47</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>7.97</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>8.76</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>7.04</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>6.34</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>4.54</t>
-        </is>
+      <c r="D9" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5.47</v>
+      </c>
+      <c r="G9" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="H9" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="I9" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="K9" t="n">
+        <v>4.54</v>
       </c>
     </row>
     <row r="10">
@@ -3491,53 +2836,35 @@
           <t>vitw_syn_noise</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="B10" t="n">
+        <v>350</v>
       </c>
       <c r="C10" t="n">
         <v>7.24</v>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>8.09</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>9.52</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>10.61</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>8.11</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>45.78</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>18.19</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>17.88</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>14.59</t>
-        </is>
+      <c r="D10" t="n">
+        <v>8.09</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="F10" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="G10" t="n">
+        <v>8.109999999999999</v>
+      </c>
+      <c r="H10" t="n">
+        <v>45.78</v>
+      </c>
+      <c r="I10" t="n">
+        <v>18.19</v>
+      </c>
+      <c r="J10" t="n">
+        <v>17.88</v>
+      </c>
+      <c r="K10" t="n">
+        <v>14.59</v>
       </c>
     </row>
     <row r="11">
@@ -3546,53 +2873,35 @@
           <t>vitw_syn_far_field</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="B11" t="n">
+        <v>350</v>
       </c>
       <c r="C11" t="n">
         <v>2.4</v>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>1.69</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>1.54</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>1.9</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>3.19</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>2.39</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>6.85</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>2.44</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>1.92</t>
-        </is>
+      <c r="D11" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="I11" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1.92</v>
       </c>
     </row>
     <row r="12">
@@ -3601,53 +2910,35 @@
           <t>vitw_syn_echo</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="B12" t="n">
+        <v>350</v>
       </c>
       <c r="C12" t="n">
         <v>11.49</v>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>12.22</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>14.61</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>14.86</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>18.21</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>28.76</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>39.87</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>32.64</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>26.58</t>
-        </is>
+      <c r="D12" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="E12" t="n">
+        <v>14.61</v>
+      </c>
+      <c r="F12" t="n">
+        <v>14.86</v>
+      </c>
+      <c r="G12" t="n">
+        <v>18.21</v>
+      </c>
+      <c r="H12" t="n">
+        <v>28.76</v>
+      </c>
+      <c r="I12" t="n">
+        <v>39.87</v>
+      </c>
+      <c r="J12" t="n">
+        <v>32.64</v>
+      </c>
+      <c r="K12" t="n">
+        <v>26.58</v>
       </c>
     </row>
     <row r="13">
@@ -3656,53 +2947,35 @@
           <t>vitw_syn_distortion</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="B13" t="n">
+        <v>350</v>
       </c>
       <c r="C13" t="n">
         <v>3.29</v>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>3.35</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>3.41</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>7.56</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>5.71</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>8.43</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>8.77</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>5.96</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>2.78</t>
-        </is>
+      <c r="D13" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="G13" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="H13" t="n">
+        <v>8.43</v>
+      </c>
+      <c r="I13" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="J13" t="n">
+        <v>5.96</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2.78</v>
       </c>
     </row>
     <row r="14">
@@ -3711,53 +2984,37 @@
           <t>vitw_syn_mixed</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>1050</t>
-        </is>
+      <c r="B14" t="n">
+        <v>1050</v>
       </c>
       <c r="C14" t="n">
         <v>4.19</v>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>4.53</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>5.39</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>9.62</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>9.29</t>
-        </is>
+      <c r="D14" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5.39</v>
+      </c>
+      <c r="F14" t="n">
+        <v>9.619999999999999</v>
+      </c>
+      <c r="G14" t="n">
+        <v>9.289999999999999</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>11.0</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>14.79</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>10.29</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>6.19</t>
-        </is>
+      <c r="I14" t="n">
+        <v>14.79</v>
+      </c>
+      <c r="J14" t="n">
+        <v>10.29</v>
+      </c>
+      <c r="K14" t="n">
+        <v>6.19</v>
       </c>
     </row>
     <row r="15">
@@ -3766,53 +3023,35 @@
           <t>vitw_syn_obstructed</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="B15" t="n">
+        <v>350</v>
       </c>
       <c r="C15" t="n">
         <v>1.97</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>1.41</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>1.27</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2.65</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>2.76</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>2.77</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>6.01</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>2.08</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>1.64</t>
-        </is>
+      <c r="D15" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="H15" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="I15" t="n">
+        <v>6.01</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.64</v>
       </c>
     </row>
     <row r="16">
@@ -3821,53 +3060,35 @@
           <t>vitw_syn_recording</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="B16" t="n">
+        <v>350</v>
       </c>
       <c r="C16" t="n">
         <v>11.55</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>13.23</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>19.42</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>19.85</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>23.33</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>22.6</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>31.81</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>30.09</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>18.09</t>
-        </is>
+      <c r="D16" t="n">
+        <v>13.23</v>
+      </c>
+      <c r="E16" t="n">
+        <v>19.42</v>
+      </c>
+      <c r="F16" t="n">
+        <v>19.85</v>
+      </c>
+      <c r="G16" t="n">
+        <v>23.33</v>
+      </c>
+      <c r="H16" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="I16" t="n">
+        <v>31.81</v>
+      </c>
+      <c r="J16" t="n">
+        <v>30.09</v>
+      </c>
+      <c r="K16" t="n">
+        <v>18.09</v>
       </c>
     </row>
     <row r="17">
@@ -3876,57 +3097,40 @@
           <t>vitw_syn_dropout</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
+      <c r="B17" t="n">
+        <v>350</v>
       </c>
       <c r="C17" t="n">
         <v>2.98</v>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>2.88</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>4.19</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>7.65</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>7.46</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>7.71</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>8.05</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>5.88</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>6.33</t>
-        </is>
+      <c r="D17" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="F17" t="n">
+        <v>7.65</v>
+      </c>
+      <c r="G17" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="H17" t="n">
+        <v>7.71</v>
+      </c>
+      <c r="I17" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="J17" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="K17" t="n">
+        <v>6.33</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -3937,7 +3141,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelRow="0"/>
+  <cols>
+    <col width="13.57142857142857" customWidth="1" min="1" max="24"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -4941,7 +4148,8 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -4951,103 +4159,195 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Lang</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>AmphionASR-1.7B</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>n</t>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Qwen3-ASR-1.7B</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Whisper-large-v3</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Kimi-Audio-7B-Instruct</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Step-Audio 2</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>MiniCPM-o</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>MOSS-Audio</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>FireRed-ASR2-LLM</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>GLM-ASR-nano</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Fun-ASR-Nano</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>whisperear_lgu_whsp</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>zh</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>CER</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="2" t="n">
+        <v>298</v>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>0.58</v>
       </c>
-      <c r="E2" t="n">
-        <v>298</v>
+      <c r="F2" s="2" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>16.33</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>15.41</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>2.75</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>whisperear_wtimit_whsp</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>WER</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="2" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>6.11</v>
       </c>
-      <c r="E3" t="n">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>aishell6_whsp</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>zh</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>CER</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>14.45</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3289</v>
+      <c r="F3" s="2" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>11.99</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>10.95</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>37.45</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>21.77</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>21.78</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>15.18</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>11.11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>